<commit_message>
pool33 v3: correct amplicon positions, off-target totals, dimer recheck, caveats
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ao75Yp9yo6KZf9ARd9UmQz
</commit_message>
<xml_diff>
--- a/docs/primer_design/primer_order_6amp_pool33_v3.xlsx
+++ b/docs/primer_design/primer_order_6amp_pool33_v3.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:A15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -501,7 +501,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>二聚体（借用 Olivar/SADDLE 打分 + primer3）：Olivar 总坏度 35447（上一版 171002，降 79%），最大单条 3385（上一版 10893）。primer3 60 °C：196×196 全部配对，全局二聚体最差 ΔG −5.4 kcal/mol（无 ≤−6 的配对），3′端锚定最差 −3.3，无严重互作。（v2 的结果；v3 的 Olivar 总坏度 35652，primer3 配对未重算，8 条延长引物仅加 1–2 nt。）</t>
+          <t>二聚体（v3 用 primer3 重算，60 °C，198 个展开序列两两）：全局最差 ΔG −5.4 kcal/mol（A3-F.1 自身），没有 ≤−6 的配对；3′端锚定最差 −3.6（A2-R.2 × A6-F.4s），没有 ≤−4 的有向配对。Olivar 总坏度 35652（v2 为 35447）。这些计算不含接头和 UDP。</t>
         </is>
       </c>
     </row>
@@ -529,7 +529,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>脱靶（新增扫描）：8 条延长引物人 ≤2 错配位点 140→14、猪 96→23，线粒体 0；双歧杆菌补充引物 A1-F.6s 人 77、猪 122 个位点（起点 20 的候选人 7、猪 15，但会命中 50% 的细菌，已弃用）。其余 24 条引物沿用 v2 的扫描结果。 v2 的整体脱靶数字（人 565 / 猪 930 位点）为 32 条版本，v3 请以订购清单逐条数字为准。</t>
+          <t>脱靶（v3 重新汇总）：人 hg19 ≤2 错配位点 516 个（v2 为 565），线粒体 ≤3 错配 0 个；潜在产物（正反向命中相距 ≤2000 bp，≤3 错配）6 个（292–1875 bp，与 v2 相同），≤2 错配 0 个。猪 susScr3 ≤2 错配位点 979 个（v2 为 930；A1-F.SNAP 占 492、新增 A1-F.6s 占 122），线粒体 0 个；≤3 错配潜在产物 18 个（v2 为 13；新增的 5 个都含 A1-F.6s，是 3 错配的正向–正向组合，342–1963 bp），≤2 错配 0 个。8 条延长引物：人 140→14 个位点，猪 96→23 个。</t>
         </is>
       </c>
     </row>
@@ -540,6 +540,16 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>重要：表中序列只是基因特异部分。你要用的 10 bp 内联 UDP（以及测序接头，如果有）必须加在 5′端，加上后的 Tm、自二聚体和管内二聚体我没有评估。订购前请把真实的 UDP 序列加到 5′端，重新跑一次二聚体检查（Olivar 的做法是把前缀计入自比对和坏度，不计入 dG）。dG ≤ −11.8 的达标比例：58 °C 时 109/198（55%），不是全部；A4 各引物、A3-R.1、A1-R.1、A5-F.1/.3、A5-R 等仍不达标：搜索 1–6 nt 延长时，没有一种延长能在位点覆盖下降不超过 0.3 个百分点的前提下达标，或延长后 J 下降超过 0.0003（A4-F.1、A4-R.4s、A5-F.3、A1-R.2、A6-F.2 属后者）。A1-F.SNAP 因 E. coli 1–8 位缺数据未延长。</t>
+        </is>
+      </c>
+    </row>
+    <row r="13"/>
+    <row r="14"/>
+    <row r="15"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3199,16 +3209,16 @@
       </c>
       <c r="D2" s="6" t="inlineStr">
         <is>
-          <t>246–265</t>
+          <t>246–266</t>
         </is>
       </c>
       <c r="E2" s="6" t="inlineStr">
         <is>
-          <t>9–264</t>
+          <t>9–266</t>
         </is>
       </c>
       <c r="F2" s="6" t="n">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="G2" s="6">
         <f>IF(F2&lt;=280,"是","基本（中间 "&amp;(F2-280)&amp;" bp 未读到）")</f>
@@ -3233,16 +3243,16 @@
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
-          <t>504–522</t>
+          <t>504–523</t>
         </is>
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>334–522</t>
+          <t>334–523</t>
         </is>
       </c>
       <c r="F3" s="6" t="n">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="G3" s="6">
         <f>IF(F3&lt;=280,"是","基本（中间 "&amp;(F3-280)&amp;" bp 未读到）")</f>
@@ -3296,21 +3306,21 @@
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>788–806</t>
+          <t>786–806</t>
         </is>
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>954–972</t>
+          <t>954–973</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>788–972</t>
+          <t>786–973</t>
         </is>
       </c>
       <c r="F5" s="6" t="n">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="G5" s="6">
         <f>IF(F5&lt;=280,"是","基本（中间 "&amp;(F5-280)&amp;" bp 未读到）")</f>
@@ -3364,21 +3374,21 @@
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>1222–1240</t>
+          <t>1220–1240</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>1486–1504</t>
+          <t>1486–1506</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>1222–1504</t>
+          <t>1220–1506</t>
         </is>
       </c>
       <c r="F7" s="6" t="n">
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="G7" s="6">
         <f>IF(F7&lt;=280,"是","基本（中间 "&amp;(F7-280)&amp;" bp 未读到）")</f>
@@ -3388,7 +3398,7 @@
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>相邻扩增子的引物位点 5′端重叠 5–6 nt（如 A3 反向 774–792 与 A4 正向 788–806），3′端不重叠，管内无短于 185 bp 的交叉产物。</t>
+          <t>相邻扩增子的引物位点 5′端重叠 5–7 nt（如 A3 反向 774–792 与 A4 正向 786–806 重叠 7 nt），3′端不重叠，管内无短于 188 bp 的交叉产物。长度为同一位点内所有引物外缘之间的最长产物，同位点内较短引物给出的产物最多短 3 bp。</t>
         </is>
       </c>
     </row>

</xml_diff>